<commit_message>
Task 6 - updated
</commit_message>
<xml_diff>
--- a/06_Operational_commercial_diagnosis/06_operational_commercial_diagnosis.xlsx
+++ b/06_Operational_commercial_diagnosis/06_operational_commercial_diagnosis.xlsx
@@ -2118,7 +2118,7 @@
         </is>
       </c>
       <c r="G3" s="6" t="n">
-        <v>-0.109</v>
+        <v>0.109</v>
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
@@ -2278,7 +2278,7 @@
         </is>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-0.102</v>
+        <v>0.102</v>
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>

</xml_diff>